<commit_message>
Fachada La Carreta: una sola puerta corrediza (vano central)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/proforma-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/proforma-fachada-la-carreta.xlsx
@@ -115,7 +115,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -130,7 +130,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precio base: $7,50 por barra (tu dato) · sobrante 24,42 m</t>
+          <t xml:space="preserve">Precio base: $7,50 por barra (tu dato) · sobrante 18,33 m</t>
         </is>
       </c>
     </row>
@@ -141,7 +141,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -169,7 +169,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -197,7 +197,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -225,7 +225,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -253,7 +253,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -276,7 +276,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -299,7 +299,7 @@
         </is>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -327,7 +327,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -350,7 +350,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -367,7 +367,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">40 en paneles + 24 bajo los rieles</t>
+          <t xml:space="preserve">40 en paneles + 8 bajo los rieles</t>
         </is>
       </c>
     </row>
@@ -378,7 +378,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -423,7 +423,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de tubo: 46,0 m², una mano</t>
+          <t xml:space="preserve">Área de tubo: 45,0 m², una mano</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mi cálculo para 620 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
+          <t xml:space="preserve">Mi cálculo para 568 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Lado) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C3">
@@ -591,7 +591,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Lado) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C4">
@@ -604,7 +604,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Lado) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C5">
@@ -617,11 +617,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Lado) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C6">
-        <v>0.7</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="7">
@@ -630,11 +630,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Lado) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C7">
-        <v>0.7</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="8">
@@ -643,11 +643,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Lado) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fijo) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C8">
-        <v>0.7</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="9">
@@ -656,11 +656,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Lado) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C9">
-        <v>0.08</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="10">
@@ -669,11 +669,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Lado) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C10">
-        <v>0.08</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="11">
@@ -682,11 +682,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Lado) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C11">
-        <v>0.08</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="12">
@@ -695,11 +695,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Lado) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C12">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="13">
@@ -708,11 +708,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Lado) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C13">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="14">
@@ -721,11 +721,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Lado) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C14">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="15">
@@ -994,7 +994,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C35">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C36">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C37">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C38">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C39">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C40">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C41">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C42">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C43">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C44">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C45">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C46">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C47">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C48">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C49">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C50">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C51">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C52">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C53">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C54">
@@ -1423,11 +1423,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,970 m (Lado) + 2 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C68">
-        <v>0.22</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="69">
@@ -1436,11 +1436,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C69">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="70">
@@ -1449,11 +1449,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C70">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="71">
@@ -1462,11 +1462,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C71">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="72">
@@ -1475,11 +1475,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C72">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="73">
@@ -1488,11 +1488,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C73">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="74">
@@ -1501,11 +1501,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C74">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="75">
@@ -1514,11 +1514,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C75">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="76">
@@ -1527,11 +1527,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C76">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="77">
@@ -1540,11 +1540,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C77">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="78">
@@ -1553,11 +1553,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C78">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="79">
@@ -1566,11 +1566,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C79">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="80">
@@ -1579,11 +1579,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C80">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="81">
@@ -1592,11 +1592,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C81">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="82">
@@ -1605,11 +1605,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C82">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="83">
@@ -1618,11 +1618,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C83">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="84">
@@ -1631,11 +1631,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C84">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="85">
@@ -1644,11 +1644,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C85">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="86">
@@ -1657,11 +1657,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C86">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="87">
@@ -1670,11 +1670,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
         </is>
       </c>
       <c r="C87">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="88">
@@ -1683,11 +1683,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">1 × 1,970 m (Lado) + 2 × 1,900 m (Puerta)</t>
         </is>
       </c>
       <c r="C88">
-        <v>0.29</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="89">
@@ -1787,11 +1787,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,900 m (Puerta) + 4 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
         </is>
       </c>
       <c r="C96">
-        <v>0.54</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="97">
@@ -1800,11 +1800,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">2 × 1,900 m (Puerta) + 2 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C97">
-        <v>0.66</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="98">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">4 × 0,888 m (Fijo) + 2 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C98">
@@ -1826,50 +1826,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 × 0,888 m (Fijo) + 4 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">4 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C99">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100">
-        <v>98</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C100">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101">
-        <v>99</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C101">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102">
-        <v>100</v>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 × 0,888 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C102">
-        <v>4.22</v>
+        <v>2.44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fachada La Carreta: cerrada por los 4 lados y desglose de tubos por lado
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/proforma-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/proforma-fachada-la-carreta.xlsx
@@ -115,7 +115,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -130,7 +130,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Precio base: $7,50 por barra (tu dato) · sobrante 10,10 m</t>
+          <t xml:space="preserve">Precio base: $7,50 por barra (tu dato) · sobrante 14,16 m</t>
         </is>
       </c>
     </row>
@@ -350,7 +350,7 @@
         </is>
       </c>
       <c r="B14">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -367,7 +367,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">16 en paneles + 8 bajo los rieles</t>
+          <t xml:space="preserve">24 en paneles + 8 bajo los rieles</t>
         </is>
       </c>
     </row>
@@ -378,7 +378,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -406,7 +406,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -423,7 +423,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de tubo: 17,9 m², una mano</t>
+          <t xml:space="preserve">Área de tubo: 35,3 m², una mano</t>
         </is>
       </c>
     </row>
@@ -434,7 +434,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -462,7 +462,7 @@
         </is>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -479,7 +479,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mi cálculo para 238 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
+          <t xml:space="preserve">Mi cálculo para 450 uniones soldadas. Con las medidas anteriores usaste 3 lb</t>
         </is>
       </c>
     </row>
@@ -578,11 +578,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Lado) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C3">
-        <v>0.7</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="4">
@@ -591,11 +591,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Lado) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C4">
-        <v>0.7</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="5">
@@ -604,11 +604,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Lado) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C5">
-        <v>0.7</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="6">
@@ -617,11 +617,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C6">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7">
@@ -630,11 +630,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C7">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="8">
@@ -643,11 +643,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C8">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="9">
@@ -656,11 +656,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C9">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="10">
@@ -669,11 +669,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C10">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="11">
@@ -682,11 +682,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C11">
-        <v>0.08</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="12">
@@ -721,7 +721,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,970 m (Fijo) + 2 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C14">
@@ -734,7 +734,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C15">
@@ -747,7 +747,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C16">
@@ -760,7 +760,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
         </is>
       </c>
       <c r="C17">
@@ -773,7 +773,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">1 × 1,970 m (Fijo) + 2 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C18">
@@ -786,7 +786,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C19">
@@ -799,7 +799,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C20">
@@ -812,7 +812,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C21">
@@ -825,7 +825,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C22">
@@ -838,7 +838,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C23">
@@ -851,7 +851,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C24">
@@ -864,7 +864,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C25">
@@ -877,7 +877,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C26">
@@ -890,7 +890,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C27">
@@ -903,7 +903,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C28">
@@ -916,7 +916,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Lado)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C29">
@@ -929,11 +929,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,970 m (Lado) + 2 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C30">
-        <v>0.22</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="31">
@@ -942,11 +942,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C31">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="32">
@@ -955,11 +955,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C32">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="33">
@@ -968,11 +968,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Der)</t>
         </is>
       </c>
       <c r="C33">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="34">
@@ -981,11 +981,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">1 × 1,970 m (Der) + 2 × 1,970 m (Izq)</t>
         </is>
       </c>
       <c r="C34">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="35">
@@ -994,11 +994,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
         </is>
       </c>
       <c r="C35">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="36">
@@ -1007,11 +1007,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
         </is>
       </c>
       <c r="C36">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="37">
@@ -1020,11 +1020,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
         </is>
       </c>
       <c r="C37">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="38">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
         </is>
       </c>
       <c r="C38">
-        <v>0.29</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="39">
@@ -1046,11 +1046,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 × 1,900 m (Puerta) + 2 × 0,888 m (Fijo)</t>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
         </is>
       </c>
       <c r="C39">
-        <v>0.41</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="40">
@@ -1059,11 +1059,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 0,888 m (Fijo) + 2 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
         </is>
       </c>
       <c r="C40">
-        <v>0.66</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="41">
@@ -1072,11 +1072,492 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">4 × 0,888 m (Puerta)</t>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
         </is>
       </c>
       <c r="C41">
-        <v>2.44</v>
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+        </is>
+      </c>
+      <c r="C42">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+        </is>
+      </c>
+      <c r="C43">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+        </is>
+      </c>
+      <c r="C44">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+        </is>
+      </c>
+      <c r="C45">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+        </is>
+      </c>
+      <c r="C46">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+        </is>
+      </c>
+      <c r="C47">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+        </is>
+      </c>
+      <c r="C48">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+        </is>
+      </c>
+      <c r="C49">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 × 1,970 m (Izq) + 2 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C50">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C51">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C52">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C53">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C54">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C55">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C56">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C57">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C58">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C59">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C60">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C61">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C62">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C63">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C64">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C65">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+        </is>
+      </c>
+      <c r="C66">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 × 1,970 m (Fondo) + 1 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C67">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C68">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C69">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C70">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C71">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C72">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C73">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>72</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C74">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C75">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>74</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C76">
+        <v>0.29</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>75</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
+        </is>
+      </c>
+      <c r="C77">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>76</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
+        </is>
+      </c>
+      <c r="C78">
+        <v>0.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fachada La Carreta: alto de 3 m
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFEggjd6XpHEYcqFvcrgyh
</commit_message>
<xml_diff>
--- a/fachada-la-carreta/proforma-fachada-la-carreta.xlsx
+++ b/fachada-la-carreta/proforma-fachada-la-carreta.xlsx
@@ -71,7 +71,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Frente 4,00 m · Alto 4,00 m · Fondo 4,00 m · Tubo 20×20 mm</t>
+          <t xml:space="preserve">Frente 4,00 m · Alto 3,00 m · Fondo 4,00 m · Tubo 20×20 mm</t>
         </is>
       </c>
     </row>
@@ -115,7 +115,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -406,7 +406,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -423,7 +423,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Área de tubo: 35,3 m², una mano</t>
+          <t xml:space="preserve">Área de tubo: 27,1 m², una mano</t>
         </is>
       </c>
     </row>
@@ -434,7 +434,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -578,11 +578,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C3">
-        <v>0.47</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="4">
@@ -591,11 +591,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C4">
-        <v>0.47</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="5">
@@ -604,11 +604,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,550 m (Fondo) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C5">
-        <v>0.47</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="6">
@@ -617,11 +617,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C6">
-        <v>0.7</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="7">
@@ -630,11 +630,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C7">
-        <v>0.7</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="8">
@@ -643,11 +643,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Der) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Fijo)</t>
         </is>
       </c>
       <c r="C8">
-        <v>0.7</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="9">
@@ -656,11 +656,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C9">
-        <v>0.7</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="10">
@@ -669,11 +669,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C10">
-        <v>0.7</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="11">
@@ -682,11 +682,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">1 × 3,325 m (Izq) + 1 × 1,470 m (Fijo) + 1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C11">
-        <v>0.7</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="12">
@@ -695,11 +695,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C12">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="13">
@@ -708,11 +708,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C13">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="14">
@@ -721,11 +721,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C14">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="15">
@@ -734,11 +734,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fijo)</t>
         </is>
       </c>
       <c r="C15">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="16">
@@ -747,11 +747,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">3 × 1,470 m (Fijo) + 1 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C16">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="17">
@@ -760,11 +760,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fijo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C17">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="18">
@@ -773,11 +773,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,970 m (Fijo) + 2 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C18">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="19">
@@ -786,11 +786,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C19">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="20">
@@ -799,11 +799,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C20">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="21">
@@ -812,11 +812,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C21">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="22">
@@ -825,11 +825,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C22">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="23">
@@ -838,11 +838,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C23">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="24">
@@ -851,11 +851,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C24">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="25">
@@ -864,11 +864,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C25">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="26">
@@ -877,11 +877,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C26">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="27">
@@ -890,11 +890,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Der)</t>
         </is>
       </c>
       <c r="C27">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="28">
@@ -903,11 +903,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">3 × 1,470 m (Der) + 1 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C28">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="29">
@@ -916,11 +916,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C29">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="30">
@@ -929,11 +929,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C30">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="31">
@@ -942,11 +942,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C31">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="32">
@@ -955,11 +955,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C32">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="33">
@@ -968,11 +968,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Der)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C33">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="34">
@@ -981,11 +981,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,970 m (Der) + 2 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C34">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="35">
@@ -994,11 +994,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C35">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="36">
@@ -1007,11 +1007,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C36">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="37">
@@ -1020,11 +1020,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C37">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="38">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C38">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="39">
@@ -1046,11 +1046,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Izq)</t>
         </is>
       </c>
       <c r="C39">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="40">
@@ -1059,11 +1059,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">3 × 1,470 m (Izq) + 1 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C40">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="41">
@@ -1072,11 +1072,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C41">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="42">
@@ -1085,11 +1085,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C42">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="43">
@@ -1098,11 +1098,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C43">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="44">
@@ -1111,11 +1111,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C44">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="45">
@@ -1124,11 +1124,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C45">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="46">
@@ -1137,11 +1137,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C46">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="47">
@@ -1150,11 +1150,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C47">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="48">
@@ -1163,11 +1163,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C48">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="49">
@@ -1176,11 +1176,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Izq)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C49">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="50">
@@ -1189,11 +1189,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 × 1,970 m (Izq) + 2 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C50">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="51">
@@ -1202,11 +1202,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C51">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="52">
@@ -1215,11 +1215,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,470 m (Fondo)</t>
         </is>
       </c>
       <c r="C52">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="53">
@@ -1228,11 +1228,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">3 × 1,470 m (Fondo) + 1 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C53">
-        <v>0.08</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="54">
@@ -1241,11 +1241,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C54">
-        <v>0.08</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="55">
@@ -1254,11 +1254,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C55">
-        <v>0.08</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="56">
@@ -1267,11 +1267,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C56">
-        <v>0.08</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="57">
@@ -1280,11 +1280,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C57">
-        <v>0.08</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="58">
@@ -1293,11 +1293,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C58">
-        <v>0.08</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="59">
@@ -1306,11 +1306,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">4 × 1,400 m (Puerta)</t>
         </is>
       </c>
       <c r="C59">
-        <v>0.08</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="60">
@@ -1319,11 +1319,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">3 × 1,400 m (Puerta) + 2 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C60">
-        <v>0.08</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="61">
@@ -1332,232 +1332,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
+          <t xml:space="preserve">1 × 0,888 m (Puerta)</t>
         </is>
       </c>
       <c r="C61">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62">
-        <v>60</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
-        </is>
-      </c>
-      <c r="C62">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63">
-        <v>61</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
-        </is>
-      </c>
-      <c r="C63">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64">
-        <v>62</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
-        </is>
-      </c>
-      <c r="C64">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65">
-        <v>63</v>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
-        </is>
-      </c>
-      <c r="C65">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66">
-        <v>64</v>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,970 m (Fondo)</t>
-        </is>
-      </c>
-      <c r="C66">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67">
-        <v>65</v>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 × 1,970 m (Fondo) + 1 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C67">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68">
-        <v>66</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C68">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69">
-        <v>67</v>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C69">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70">
-        <v>68</v>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C70">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71">
-        <v>69</v>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C71">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72">
-        <v>70</v>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C72">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73">
-        <v>71</v>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C73">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74">
-        <v>72</v>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C74">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75">
-        <v>73</v>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C75">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76">
-        <v>74</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 × 1,900 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C76">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77">
-        <v>75</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 × 0,888 m (Fijo)</t>
-        </is>
-      </c>
-      <c r="C77">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78">
-        <v>76</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6 × 0,888 m (Puerta)</t>
-        </is>
-      </c>
-      <c r="C78">
-        <v>0.66</v>
+        <v>5.11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>